<commit_message>
Peter brief xlsx: clickable-GIF requirements + CapCut/ffmpeg method
</commit_message>
<xml_diff>
--- a/build-specs/Peter_New_Leads_Content_Brief.xlsx
+++ b/build-specs/Peter_New_Leads_Content_Brief.xlsx
@@ -94,9 +94,7 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -481,22 +479,22 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="46" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Peter — New Leads Pipeline Content Brief (videos + captioned GIFs)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="58" customHeight="1">
+          <t>Peter — New Leads Pipeline Content Brief (videos + clickable GIFs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="78" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HOW THIS WORKS: For every video you make, also export a 3 to 4 second SILENT GIF clipped from it, with the caption text below burned onto the GIF. The GIF is what gets texted/emailed; tapping it opens the page where the full video plays. Lipdub = personalized (name swaps per lead). Static = no name, reusable at scale. Build draft assets; John wires them into GHL after.</t>
+          <t>HOW THIS WORKS: For each video, also export the GIF that gets texted/emailed. A plain link looks like spam, so every GIF must be a 3-4 second silent loop with (1) a PLAY-BUTTON overlay and (2) a bold 'TAP TO WATCH' cue burned across the bottom, plus the caption below. Lipdub makes its personalized GIFs automatically (you do NOT make those). For static/testimonial/HeyGen videos, make the GIF in CapCut (clip + play-button sticker + 'TAP TO WATCH'), or hand videos to the team to batch-generate. Build draft assets; John wires them into GHL after.</t>
         </is>
       </c>
     </row>
@@ -538,7 +536,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>GIF caption (burn this onto the GIF)</t>
+          <t>GIF caption (burn on, end with TAP TO WATCH)</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -552,7 +550,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="58" customHeight="1">
+    <row r="4" ht="60" customHeight="1">
       <c r="A4" s="4" t="n">
         <v>1</v>
       </c>
@@ -588,12 +586,12 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Tried to reach you about your home search. Tap to watch.</t>
+          <t>Tried to reach you about your home search. TAP TO WATCH.</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Full script in pipeline dashboard. Goes out as VM + GIF MMS.</t>
+          <t>Lipdub auto-makes the GIF + landing page. Full script in dashboard.</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -602,7 +600,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>2</v>
       </c>
@@ -633,17 +631,17 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Same as above, selfie at eye level, name swap, point to link, wave.</t>
+          <t>Same selfie shot, name swap, point to link, wave.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Tried to reach you about your property. Tap to watch.</t>
+          <t>Tried to reach you about your property. TAP TO WATCH.</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Seller version of the Day 1 intro.</t>
+          <t>Lipdub auto-makes the GIF.</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -652,7 +650,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="58" customHeight="1">
+    <row r="6" ht="60" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>3</v>
       </c>
@@ -688,12 +686,12 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Glad you reached out. Here's how I help. Tap to watch.</t>
+          <t>Glad you reached out. Here's how I help. TAP TO WATCH.</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>For leads who replied. Generic (works buyer or seller).</t>
+          <t>Lipdub auto-makes the GIF. Works buyer or seller.</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -702,7 +700,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="58" customHeight="1">
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>4</v>
       </c>
@@ -733,17 +731,17 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Vertical, no name (reusable at scale). Talk to camera ~15-20s, friendly, plain background.</t>
+          <t>Vertical, no name (reusable). ~15-20s to camera, plain background.</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>How I help buyers in your area. Tap to watch.</t>
+          <t>How I help buyers in your area. TAP TO WATCH.</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Reused later in Email/Text-Only and Cold stages too.</t>
+          <t>Make GIF in CapCut: clip + play-button + TAP TO WATCH. Reused in Email/Text-Only + Cold.</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -752,7 +750,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="58" customHeight="1">
+    <row r="8" ht="60" customHeight="1">
       <c r="A8" s="4" t="n">
         <v>5</v>
       </c>
@@ -788,12 +786,12 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>How I help sellers in your area. Tap to watch.</t>
+          <t>How I help sellers in your area. TAP TO WATCH.</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Reused in Email/Text-Only and Cold stages.</t>
+          <t>CapCut GIF with overlay. Reused in Email/Text-Only + Cold.</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -802,7 +800,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="58" customHeight="1">
+    <row r="9" ht="60" customHeight="1">
       <c r="A9" s="4" t="n">
         <v>6</v>
       </c>
@@ -833,17 +831,17 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Vertical, no name. Short story of helping a buyer win.</t>
+          <t>Vertical, no name. Short buyer-win story.</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>How I've helped buyers land the right home. Tap to watch.</t>
+          <t>How I've helped buyers land the right home. TAP TO WATCH.</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Can reuse an existing buyer win clip if you have one.</t>
+          <t>CapCut GIF with overlay. Reuse existing clip if available.</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -852,7 +850,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="58" customHeight="1">
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" s="4" t="n">
         <v>7</v>
       </c>
@@ -883,17 +881,17 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Vertical, no name. Short story of a strong seller result.</t>
+          <t>Vertical, no name. Short strong-result story.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>How I've helped sellers get a strong result. Tap to watch.</t>
+          <t>How I've helped sellers get a strong result. TAP TO WATCH.</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Reuse existing if available.</t>
+          <t>CapCut GIF with overlay. Reuse existing if available.</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -902,7 +900,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="58" customHeight="1">
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="4" t="n">
         <v>8</v>
       </c>
@@ -933,17 +931,17 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Client on camera if possible, or Graeham telling the story. Vertical.</t>
+          <t>Client on camera if possible, or Graeham narrating. Vertical.</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>How a buyer like you found the right home. Tap to watch.</t>
+          <t>How a buyer like you found the right home. TAP TO WATCH.</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Use an existing testimonial if we already have a buyer one.</t>
+          <t>CapCut GIF with overlay. Use existing buyer testimonial if we have one.</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -952,7 +950,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="58" customHeight="1">
+    <row r="12" ht="60" customHeight="1">
       <c r="A12" s="4" t="n">
         <v>9</v>
       </c>
@@ -988,12 +986,12 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>How a seller like you got a strong result. Tap to watch.</t>
+          <t>How a seller like you got a strong result. TAP TO WATCH.</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Use existing seller testimonial if available.</t>
+          <t>CapCut GIF with overlay. Use existing seller testimonial if available.</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1002,7 +1000,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="58" customHeight="1">
+    <row r="13" ht="60" customHeight="1">
       <c r="A13" s="4" t="n">
         <v>10</v>
       </c>
@@ -1033,7 +1031,7 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>No new filming. We reuse your latest weekly market update video.</t>
+          <t>No filming. Reuse the latest weekly market update video.</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1043,7 +1041,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Just confirm the newest market video is embedded at graehamwatts.com/the-bay-real-estate-market or top of the YouTube Videos tab.</t>
+          <t>Confirm newest market video is embedded at graehamwatts.com/the-bay-real-estate-market or top of YouTube Videos tab.</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1052,13 +1050,13 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="58" customHeight="1">
+    <row r="14" ht="60" customHeight="1">
       <c r="A14" s="4" t="n">
         <v>11</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Market update (HeyGen option)</t>
+          <t>Market explainer (HeyGen)</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1083,17 +1081,17 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>AI avatar video (generated, no filming). Only if we want a fresh market explainer for the long-cadence stages.</t>
+          <t>AI avatar video (generated, no filming). Optional fresh market explainer for long-cadence stages.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Market video. Tap to watch.</t>
+          <t>Market video. TAP TO WATCH.</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Optional. Reuse existing market content where possible.</t>
+          <t>If used, make GIF with overlay. Reuse existing market content where possible.</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">

</xml_diff>